<commit_message>
fixed heatmap for non-96 well plates, fixed sizing of text on plate map and demultiplexed plots, implemented plan to ask user to overwrite output directory at start of pipeline, fixed a few BIN miscalculations in final html file (7b), added paired end option to command line, rather than parameters file
</commit_message>
<xml_diff>
--- a/Docker/parameters.xlsx
+++ b/Docker/parameters.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickbard/Desktop/CBG/MAP/Docker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A4A4081-A810-364A-A6A5-385D5C397F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{196D9DF5-5848-AD48-B698-696A65157FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="30240" windowHeight="16320" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="362">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="361">
   <si>
     <t xml:space="preserve">NOTE: Parameters in red are mandatory </t>
   </si>
@@ -1154,9 +1154,6 @@
   </si>
   <si>
     <t>Min Reads per OTU</t>
-  </si>
-  <si>
-    <t>No</t>
   </si>
   <si>
     <t>Dictionary Update</t>
@@ -2056,7 +2053,7 @@
         <v>38</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
@@ -2065,7 +2062,7 @@
         <v>39</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -2140,7 +2137,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="32" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="30"/>
@@ -2151,7 +2148,7 @@
         <v>38</v>
       </c>
       <c r="C23" s="35" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
@@ -2160,7 +2157,7 @@
         <v>39</v>
       </c>
       <c r="C24" s="35" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
@@ -2202,7 +2199,7 @@
     <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="31"/>
       <c r="B29" s="34" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C29" s="35" t="s">
         <v>21</v>
@@ -2211,7 +2208,7 @@
     <row r="30" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="31"/>
       <c r="B30" s="34" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C30" s="35" t="s">
         <v>22</v>
@@ -2220,7 +2217,7 @@
     <row r="31" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="31"/>
       <c r="B31" s="34" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C31" s="35" t="s">
         <v>23</v>
@@ -2229,7 +2226,7 @@
     <row r="32" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="31"/>
       <c r="B32" s="34" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C32" s="35" t="s">
         <v>3</v>
@@ -2247,7 +2244,7 @@
     <row r="34" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="31"/>
       <c r="B34" s="34" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C34" s="35" t="s">
         <v>4</v>
@@ -2256,7 +2253,7 @@
     <row r="35" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="31"/>
       <c r="B35" s="34" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C35" s="35" t="s">
         <v>341</v>
@@ -2265,7 +2262,7 @@
     <row r="36" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="31"/>
       <c r="B36" s="34" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C36" s="35" t="s">
         <v>342</v>
@@ -7666,7 +7663,7 @@
   <sheetPr>
     <tabColor rgb="FFFF3838"/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="14.33203125" customWidth="1"/>
@@ -7676,7 +7673,7 @@
     <col min="6" max="6" width="30.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="48" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:13" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="12" t="s">
         <v>38</v>
       </c>
@@ -7696,19 +7693,19 @@
         <v>24</v>
       </c>
       <c r="G1" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="H1" s="18" t="s">
         <v>354</v>
       </c>
-      <c r="H1" s="18" t="s">
+      <c r="I1" s="18" t="s">
         <v>355</v>
       </c>
-      <c r="I1" s="18" t="s">
-        <v>356</v>
-      </c>
       <c r="J1" s="29" t="s">
+        <v>347</v>
+      </c>
+      <c r="K1" s="29" t="s">
         <v>357</v>
-      </c>
-      <c r="K1" s="29" t="s">
-        <v>347</v>
       </c>
       <c r="L1" s="29" t="s">
         <v>358</v>
@@ -7716,11 +7713,8 @@
       <c r="M1" s="29" t="s">
         <v>359</v>
       </c>
-      <c r="N1" s="29" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>45</v>
       </c>
@@ -7737,7 +7731,7 @@
         <v>338</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="G2" s="19">
         <v>640</v>
@@ -7748,19 +7742,16 @@
       <c r="I2" s="19">
         <v>658</v>
       </c>
-      <c r="J2" s="14" t="s">
-        <v>348</v>
+      <c r="J2" s="19">
+        <v>3</v>
       </c>
       <c r="K2" s="19">
-        <v>3</v>
-      </c>
-      <c r="L2" s="19">
         <v>8</v>
       </c>
+      <c r="L2" s="14">
+        <v>5</v>
+      </c>
       <c r="M2" s="14">
-        <v>5</v>
-      </c>
-      <c r="N2" s="14">
         <v>2.2999999999999998</v>
       </c>
     </row>

</xml_diff>

<commit_message>
clarified points on README, made parameters files that do not include paired-end read tab and allow for Reverse Complementation of certain primer sets, edited compose.yaml so it can handle datasets with many wells
</commit_message>
<xml_diff>
--- a/Docker/parameters.xlsx
+++ b/Docker/parameters.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickbard/Desktop/CBG/MAP/Docker/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{196D9DF5-5848-AD48-B698-696A65157FD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{945E5A91-9223-0F4F-B9E0-EE9C4E2C10DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="30240" windowHeight="16320" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-31480" yWindow="4200" windowWidth="30240" windowHeight="16320" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="362">
   <si>
     <t xml:space="preserve">NOTE: Parameters in red are mandatory </t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>The name of your sequencing run.</t>
-  </si>
-  <si>
-    <t>Whether or not your input reads will be paired-end (Illumina R1 and R2 fastq files) or not (one or more regular fastq files).</t>
   </si>
   <si>
     <t xml:space="preserve">The number of replicates per sample used. </t>
@@ -1180,9 +1177,6 @@
     <t>Target Amplicon Length</t>
   </si>
   <si>
-    <t>Paired-End Reads</t>
-  </si>
-  <si>
     <t>Replicates per Sample</t>
   </si>
   <si>
@@ -1193,6 +1187,15 @@
   </si>
   <si>
     <t>BOLDistilled_COI_</t>
+  </si>
+  <si>
+    <t>Reverse Complement</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Default is 'No' or [blank] and it is unlikely that you will need to change this. Set 'Yes' only for a primer row with reads that come off the sequencer starting from the reverse-primer end (e.g., plates built with the layout reversed so UMIs can be reused). That row's primer sequences must also be entered swapped (the reverse primer in the Forward Primer Sequence column).</t>
   </si>
 </sst>
 </file>
@@ -1319,7 +1322,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1440,6 +1443,12 @@
         <bgColor rgb="FF800080"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="65"/>
+        <bgColor theme="0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -1479,7 +1488,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1559,6 +1568,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="15" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1974,7 +1987,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="21" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
@@ -1988,7 +2001,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -2005,78 +2018,78 @@
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="B5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="B6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>7</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="B7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="4" t="s">
         <v>9</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
       <c r="B8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
       <c r="B9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
       <c r="B10" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
       <c r="B11" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
       <c r="B12" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -2084,60 +2097,60 @@
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="7"/>
       <c r="B15" s="24" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="7"/>
       <c r="B16" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="25" t="s">
         <v>28</v>
-      </c>
-      <c r="C16" s="25" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="7"/>
       <c r="B17" s="24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="25" t="s">
         <v>30</v>
-      </c>
-      <c r="C17" s="25" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="7"/>
       <c r="B18" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="25" t="s">
         <v>32</v>
-      </c>
-      <c r="C18" s="25" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="7"/>
       <c r="B19" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="25" t="s">
         <v>34</v>
-      </c>
-      <c r="C19" s="25" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="7"/>
       <c r="B20" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C20" s="25" t="s">
         <v>36</v>
-      </c>
-      <c r="C20" s="25" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="32" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="30"/>
@@ -2145,115 +2158,115 @@
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="30"/>
       <c r="B23" s="33" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C23" s="35" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="30"/>
       <c r="B24" s="33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C24" s="35" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="31"/>
       <c r="B25" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="C25" s="35" t="s">
         <v>11</v>
-      </c>
-      <c r="C25" s="35" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="31"/>
       <c r="B26" s="33" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="35" t="s">
         <v>13</v>
-      </c>
-      <c r="C26" s="35" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="31"/>
       <c r="B27" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="35" t="s">
         <v>19</v>
-      </c>
-      <c r="C27" s="35" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="31"/>
       <c r="B28" s="34" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" s="35" t="s">
         <v>24</v>
-      </c>
-      <c r="C28" s="35" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="31"/>
       <c r="B29" s="34" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C29" s="35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="31"/>
       <c r="B30" s="34" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C30" s="35" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="31"/>
       <c r="B31" s="34" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C31" s="35" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="31"/>
       <c r="B32" s="34" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
       <c r="C32" s="35" t="s">
-        <v>3</v>
+        <v>339</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="31"/>
       <c r="B33" s="34" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="C33" s="35" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="31"/>
       <c r="B34" s="34" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="C34" s="35" t="s">
-        <v>4</v>
+        <v>340</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="31"/>
       <c r="B35" s="34" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C35" s="35" t="s">
         <v>341</v>
@@ -2264,13 +2277,18 @@
       <c r="B36" s="34" t="s">
         <v>359</v>
       </c>
-      <c r="C36" s="35" t="s">
-        <v>342</v>
-      </c>
+      <c r="C36" s="38" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" s="37" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A37"/>
+      <c r="B37"/>
+      <c r="C37"/>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C38" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -2305,7 +2323,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C1" s="28"/>
       <c r="D1" s="22"/>
@@ -2320,2345 +2338,2345 @@
     </row>
     <row r="2" spans="1:12" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F2" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="G2" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="H2" s="13" t="s">
         <v>39</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="C3" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="D3" t="s">
         <v>43</v>
       </c>
-      <c r="D3" t="s">
-        <v>44</v>
-      </c>
       <c r="E3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H3" s="14"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="D4" t="s">
         <v>48</v>
       </c>
-      <c r="D4" t="s">
-        <v>49</v>
-      </c>
       <c r="E4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H4" s="14"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="D5" t="s">
         <v>51</v>
       </c>
-      <c r="D5" t="s">
-        <v>52</v>
-      </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H5" s="14"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="D6" t="s">
         <v>54</v>
       </c>
-      <c r="D6" t="s">
-        <v>55</v>
-      </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H6" s="14"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" t="s">
         <v>57</v>
       </c>
-      <c r="D7" t="s">
-        <v>58</v>
-      </c>
       <c r="E7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H7" s="14"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="14" t="s">
+      <c r="D8" t="s">
         <v>60</v>
       </c>
-      <c r="D8" t="s">
-        <v>61</v>
-      </c>
       <c r="E8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H8" s="14"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C9" s="14" t="s">
+      <c r="D9" t="s">
         <v>63</v>
       </c>
-      <c r="D9" t="s">
-        <v>64</v>
-      </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H9" s="14"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="D10" t="s">
         <v>66</v>
       </c>
-      <c r="D10" t="s">
-        <v>67</v>
-      </c>
       <c r="E10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H10" s="14"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B11" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="D11" t="s">
         <v>69</v>
       </c>
-      <c r="D11" t="s">
-        <v>70</v>
-      </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H11" s="14"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B12" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C12" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="D12" t="s">
         <v>72</v>
       </c>
-      <c r="D12" t="s">
-        <v>73</v>
-      </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H12" s="14"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C13" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="D13" t="s">
         <v>75</v>
       </c>
-      <c r="D13" t="s">
-        <v>76</v>
-      </c>
       <c r="E13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H13" s="14"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B14" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="C14" s="14" t="s">
+      <c r="D14" t="s">
         <v>78</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E14" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="H14" s="14" t="s">
         <v>79</v>
-      </c>
-      <c r="E14" t="s">
-        <v>79</v>
-      </c>
-      <c r="F14" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G14" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B15" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="D15" t="s">
         <v>82</v>
       </c>
-      <c r="D15" t="s">
-        <v>83</v>
-      </c>
       <c r="E15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G15" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H15" s="14"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B16" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="D16" t="s">
         <v>85</v>
       </c>
-      <c r="D16" t="s">
-        <v>86</v>
-      </c>
       <c r="E16" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G16" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H16" s="14"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B17" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="C17" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="D17" t="s">
         <v>88</v>
       </c>
-      <c r="D17" t="s">
-        <v>89</v>
-      </c>
       <c r="E17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G17" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H17" s="14"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="14" t="s">
+      <c r="D18" t="s">
         <v>91</v>
       </c>
-      <c r="D18" t="s">
-        <v>92</v>
-      </c>
       <c r="E18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F18" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G18" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H18" s="14"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="C19" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="C19" s="14" t="s">
+      <c r="D19" t="s">
         <v>94</v>
       </c>
-      <c r="D19" t="s">
-        <v>95</v>
-      </c>
       <c r="E19" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F19" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G19" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H19" s="14"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B20" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="C20" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="C20" s="14" t="s">
+      <c r="D20" t="s">
         <v>97</v>
       </c>
-      <c r="D20" t="s">
-        <v>98</v>
-      </c>
       <c r="E20" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F20" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G20" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H20" s="14"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="C21" s="14" t="s">
         <v>99</v>
       </c>
-      <c r="C21" s="14" t="s">
+      <c r="D21" t="s">
         <v>100</v>
       </c>
-      <c r="D21" t="s">
-        <v>101</v>
-      </c>
       <c r="E21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F21" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G21" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H21" s="14"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B22" s="14" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" s="14" t="s">
         <v>102</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="D22" t="s">
         <v>103</v>
       </c>
-      <c r="D22" t="s">
-        <v>104</v>
-      </c>
       <c r="E22" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F22" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G22" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H22" s="14"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B23" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="C23" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="C23" s="14" t="s">
+      <c r="D23" t="s">
         <v>106</v>
       </c>
-      <c r="D23" t="s">
-        <v>107</v>
-      </c>
       <c r="E23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H23" s="14"/>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B24" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C24" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="C24" s="14" t="s">
+      <c r="D24" t="s">
         <v>109</v>
       </c>
-      <c r="D24" t="s">
-        <v>110</v>
-      </c>
       <c r="E24" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H24" s="14"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B25" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="C25" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="C25" s="14" t="s">
+      <c r="D25" t="s">
         <v>112</v>
       </c>
-      <c r="D25" t="s">
-        <v>113</v>
-      </c>
       <c r="E25" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F25" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G25" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H25" s="14"/>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B26" s="14" t="s">
+        <v>113</v>
+      </c>
+      <c r="C26" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="D26" t="s">
         <v>115</v>
       </c>
-      <c r="D26" t="s">
-        <v>116</v>
-      </c>
       <c r="E26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F26" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G26" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B27" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="C27" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C27" s="14" t="s">
+      <c r="D27" t="s">
         <v>118</v>
       </c>
-      <c r="D27" t="s">
-        <v>119</v>
-      </c>
       <c r="E27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F27" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G27" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H27" s="14"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B28" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="C28" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="C28" s="14" t="s">
+      <c r="D28" t="s">
         <v>121</v>
       </c>
-      <c r="D28" t="s">
-        <v>122</v>
-      </c>
       <c r="E28" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H28" s="14"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B29" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="C29" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="D29" t="s">
         <v>124</v>
       </c>
-      <c r="D29" t="s">
-        <v>125</v>
-      </c>
       <c r="E29" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F29" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G29" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H29" s="14"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B30" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C30" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="D30" t="s">
         <v>127</v>
       </c>
-      <c r="D30" t="s">
-        <v>128</v>
-      </c>
       <c r="E30" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G30" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H30" s="14"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="C31" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="C31" s="14" t="s">
+      <c r="D31" t="s">
         <v>130</v>
       </c>
-      <c r="D31" t="s">
-        <v>131</v>
-      </c>
       <c r="E31" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H31" s="14"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B32" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="D32" t="s">
         <v>133</v>
       </c>
-      <c r="D32" t="s">
-        <v>134</v>
-      </c>
       <c r="E32" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F32" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G32" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H32" s="14"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B33" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="C33" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="C33" s="14" t="s">
+      <c r="D33" t="s">
         <v>136</v>
       </c>
-      <c r="D33" t="s">
-        <v>137</v>
-      </c>
       <c r="E33" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H33" s="14"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B34" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="C34" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="C34" s="14" t="s">
+      <c r="D34" t="s">
         <v>139</v>
       </c>
-      <c r="D34" t="s">
-        <v>140</v>
-      </c>
       <c r="E34" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H34" s="14"/>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B35" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="C35" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="C35" s="14" t="s">
+      <c r="D35" t="s">
         <v>142</v>
       </c>
-      <c r="D35" t="s">
-        <v>143</v>
-      </c>
       <c r="E35" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H35" s="14"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B36" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="C36" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="C36" s="14" t="s">
+      <c r="D36" t="s">
         <v>145</v>
       </c>
-      <c r="D36" t="s">
-        <v>146</v>
-      </c>
       <c r="E36" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H36" s="14"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B37" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="C37" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="C37" s="14" t="s">
+      <c r="D37" t="s">
         <v>148</v>
       </c>
-      <c r="D37" t="s">
-        <v>149</v>
-      </c>
       <c r="E37" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H37" s="14"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B38" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="C38" s="14" t="s">
         <v>150</v>
       </c>
-      <c r="C38" s="14" t="s">
+      <c r="D38" t="s">
         <v>151</v>
       </c>
-      <c r="D38" t="s">
-        <v>152</v>
-      </c>
       <c r="E38" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B39" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="C39" s="14" t="s">
+      <c r="D39" t="s">
         <v>154</v>
       </c>
-      <c r="D39" t="s">
-        <v>155</v>
-      </c>
       <c r="E39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F39" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H39" s="14"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B40" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="C40" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="C40" s="14" t="s">
+      <c r="D40" t="s">
         <v>157</v>
       </c>
-      <c r="D40" t="s">
-        <v>158</v>
-      </c>
       <c r="E40" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G40" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H40" s="14"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="C41" s="14" t="s">
+      <c r="D41" t="s">
         <v>160</v>
       </c>
-      <c r="D41" t="s">
-        <v>161</v>
-      </c>
       <c r="E41" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F41" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G41" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H41" s="14"/>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="C42" s="14" t="s">
         <v>162</v>
       </c>
-      <c r="C42" s="14" t="s">
+      <c r="D42" t="s">
         <v>163</v>
       </c>
-      <c r="D42" t="s">
-        <v>164</v>
-      </c>
       <c r="E42" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F42" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G42" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H42" s="14"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B43" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C43" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="C43" s="14" t="s">
+      <c r="D43" t="s">
         <v>166</v>
       </c>
-      <c r="D43" t="s">
-        <v>167</v>
-      </c>
       <c r="E43" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G43" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H43" s="14"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B44" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="C44" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="C44" s="14" t="s">
+      <c r="D44" t="s">
         <v>169</v>
       </c>
-      <c r="D44" t="s">
-        <v>170</v>
-      </c>
       <c r="E44" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G44" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H44" s="14"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B45" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="C45" s="14" t="s">
         <v>171</v>
       </c>
-      <c r="C45" s="14" t="s">
+      <c r="D45" t="s">
         <v>172</v>
       </c>
-      <c r="D45" t="s">
-        <v>173</v>
-      </c>
       <c r="E45" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F45" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H45" s="14"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A46" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B46" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="C46" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="C46" s="14" t="s">
+      <c r="D46" t="s">
         <v>175</v>
       </c>
-      <c r="D46" t="s">
-        <v>176</v>
-      </c>
       <c r="E46" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F46" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G46" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H46" s="14"/>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A47" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B47" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="C47" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="C47" s="14" t="s">
+      <c r="D47" t="s">
         <v>178</v>
       </c>
-      <c r="D47" t="s">
-        <v>179</v>
-      </c>
       <c r="E47" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F47" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G47" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H47" s="14"/>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B48" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="C48" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="C48" s="14" t="s">
+      <c r="D48" t="s">
         <v>181</v>
       </c>
-      <c r="D48" t="s">
-        <v>182</v>
-      </c>
       <c r="E48" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G48" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H48" s="14"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B49" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="C49" s="14" t="s">
         <v>183</v>
       </c>
-      <c r="C49" s="14" t="s">
+      <c r="D49" t="s">
         <v>184</v>
       </c>
-      <c r="D49" t="s">
-        <v>185</v>
-      </c>
       <c r="E49" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F49" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G49" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H49" s="14"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B50" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="C50" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="C50" s="14" t="s">
+      <c r="D50" t="s">
         <v>187</v>
       </c>
-      <c r="D50" t="s">
-        <v>188</v>
-      </c>
       <c r="E50" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F50" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G50" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H50" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B51" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="C51" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="C51" s="14" t="s">
+      <c r="D51" t="s">
         <v>190</v>
       </c>
-      <c r="D51" t="s">
-        <v>191</v>
-      </c>
       <c r="E51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F51" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G51" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H51" s="14"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B52" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="C52" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="C52" s="14" t="s">
+      <c r="D52" t="s">
         <v>193</v>
       </c>
-      <c r="D52" t="s">
-        <v>194</v>
-      </c>
       <c r="E52" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F52" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G52" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H52" s="14"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B53" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="C53" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="C53" s="14" t="s">
+      <c r="D53" t="s">
         <v>196</v>
       </c>
-      <c r="D53" t="s">
-        <v>197</v>
-      </c>
       <c r="E53" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F53" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G53" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H53" s="14"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B54" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="C54" s="14" t="s">
         <v>198</v>
       </c>
-      <c r="C54" s="14" t="s">
+      <c r="D54" t="s">
         <v>199</v>
       </c>
-      <c r="D54" t="s">
-        <v>200</v>
-      </c>
       <c r="E54" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F54" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G54" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H54" s="14"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B55" s="14" t="s">
+        <v>200</v>
+      </c>
+      <c r="C55" s="14" t="s">
         <v>201</v>
       </c>
-      <c r="C55" s="14" t="s">
+      <c r="D55" t="s">
         <v>202</v>
       </c>
-      <c r="D55" t="s">
-        <v>203</v>
-      </c>
       <c r="E55" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F55" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G55" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H55" s="14"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B56" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="C56" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="C56" s="14" t="s">
+      <c r="D56" t="s">
         <v>205</v>
       </c>
-      <c r="D56" t="s">
-        <v>206</v>
-      </c>
       <c r="E56" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F56" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G56" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H56" s="14"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B57" s="14" t="s">
+        <v>206</v>
+      </c>
+      <c r="C57" s="14" t="s">
         <v>207</v>
       </c>
-      <c r="C57" s="14" t="s">
+      <c r="D57" t="s">
         <v>208</v>
       </c>
-      <c r="D57" t="s">
-        <v>209</v>
-      </c>
       <c r="E57" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F57" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G57" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H57" s="14"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A58" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B58" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="C58" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="C58" s="14" t="s">
+      <c r="D58" t="s">
         <v>211</v>
       </c>
-      <c r="D58" t="s">
-        <v>212</v>
-      </c>
       <c r="E58" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F58" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G58" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H58" s="14"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A59" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B59" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="C59" s="14" t="s">
         <v>213</v>
       </c>
-      <c r="C59" s="14" t="s">
+      <c r="D59" t="s">
         <v>214</v>
       </c>
-      <c r="D59" t="s">
-        <v>215</v>
-      </c>
       <c r="E59" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F59" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G59" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H59" s="14"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B60" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="C60" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="C60" s="14" t="s">
+      <c r="D60" t="s">
         <v>217</v>
       </c>
-      <c r="D60" t="s">
-        <v>218</v>
-      </c>
       <c r="E60" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F60" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G60" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H60" s="14"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B61" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="C61" s="14" t="s">
         <v>219</v>
       </c>
-      <c r="C61" s="14" t="s">
+      <c r="D61" t="s">
         <v>220</v>
       </c>
-      <c r="D61" t="s">
-        <v>221</v>
-      </c>
       <c r="E61" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F61" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G61" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H61" s="14"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B62" s="14" t="s">
+        <v>221</v>
+      </c>
+      <c r="C62" s="14" t="s">
         <v>222</v>
       </c>
-      <c r="C62" s="14" t="s">
+      <c r="D62" t="s">
         <v>223</v>
       </c>
-      <c r="D62" t="s">
-        <v>224</v>
-      </c>
       <c r="E62" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G62" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H62" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B63" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="C63" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="C63" s="14" t="s">
+      <c r="D63" t="s">
         <v>226</v>
       </c>
-      <c r="D63" t="s">
-        <v>227</v>
-      </c>
       <c r="E63" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F63" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G63" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H63" s="14"/>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B64" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="C64" s="14" t="s">
         <v>228</v>
       </c>
-      <c r="C64" s="14" t="s">
+      <c r="D64" t="s">
         <v>229</v>
       </c>
-      <c r="D64" t="s">
-        <v>230</v>
-      </c>
       <c r="E64" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F64" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G64" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H64" s="14"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B65" s="14" t="s">
+        <v>230</v>
+      </c>
+      <c r="C65" s="14" t="s">
         <v>231</v>
       </c>
-      <c r="C65" s="14" t="s">
+      <c r="D65" t="s">
         <v>232</v>
       </c>
-      <c r="D65" t="s">
-        <v>233</v>
-      </c>
       <c r="E65" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F65" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G65" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H65" s="14"/>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B66" s="14" t="s">
+        <v>233</v>
+      </c>
+      <c r="C66" s="14" t="s">
         <v>234</v>
       </c>
-      <c r="C66" s="14" t="s">
+      <c r="D66" t="s">
         <v>235</v>
       </c>
-      <c r="D66" t="s">
-        <v>236</v>
-      </c>
       <c r="E66" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F66" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G66" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H66" s="14"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B67" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="C67" s="14" t="s">
         <v>237</v>
       </c>
-      <c r="C67" s="14" t="s">
+      <c r="D67" t="s">
         <v>238</v>
       </c>
-      <c r="D67" t="s">
-        <v>239</v>
-      </c>
       <c r="E67" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F67" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G67" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H67" s="14"/>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A68" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B68" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="C68" s="14" t="s">
         <v>240</v>
       </c>
-      <c r="C68" s="14" t="s">
+      <c r="D68" t="s">
         <v>241</v>
       </c>
-      <c r="D68" t="s">
-        <v>242</v>
-      </c>
       <c r="E68" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F68" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G68" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H68" s="14"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B69" s="14" t="s">
+        <v>242</v>
+      </c>
+      <c r="C69" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="C69" s="14" t="s">
+      <c r="D69" t="s">
         <v>244</v>
       </c>
-      <c r="D69" t="s">
-        <v>245</v>
-      </c>
       <c r="E69" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F69" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G69" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H69" s="14"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B70" s="14" t="s">
+        <v>245</v>
+      </c>
+      <c r="C70" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="C70" s="14" t="s">
+      <c r="D70" t="s">
         <v>247</v>
       </c>
-      <c r="D70" t="s">
-        <v>248</v>
-      </c>
       <c r="E70" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="F70" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G70" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H70" s="14"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B71" s="14" t="s">
+        <v>248</v>
+      </c>
+      <c r="C71" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="C71" s="14" t="s">
+      <c r="D71" t="s">
         <v>250</v>
       </c>
-      <c r="D71" t="s">
-        <v>251</v>
-      </c>
       <c r="E71" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F71" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G71" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H71" s="14"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B72" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="C72" s="14" t="s">
         <v>252</v>
       </c>
-      <c r="C72" s="14" t="s">
+      <c r="D72" t="s">
         <v>253</v>
       </c>
-      <c r="D72" t="s">
-        <v>254</v>
-      </c>
       <c r="E72" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="F72" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G72" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H72" s="14"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B73" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="C73" s="14" t="s">
         <v>255</v>
       </c>
-      <c r="C73" s="14" t="s">
+      <c r="D73" t="s">
         <v>256</v>
       </c>
-      <c r="D73" t="s">
-        <v>257</v>
-      </c>
       <c r="E73" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="F73" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G73" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H73" s="14"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A74" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B74" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="C74" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="C74" s="14" t="s">
+      <c r="D74" t="s">
         <v>259</v>
       </c>
-      <c r="D74" t="s">
-        <v>260</v>
-      </c>
       <c r="E74" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="F74" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G74" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H74" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B75" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="C75" s="14" t="s">
         <v>261</v>
       </c>
-      <c r="C75" s="14" t="s">
+      <c r="D75" t="s">
         <v>262</v>
       </c>
-      <c r="D75" t="s">
-        <v>263</v>
-      </c>
       <c r="E75" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="F75" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G75" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H75" s="14"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B76" s="14" t="s">
+        <v>263</v>
+      </c>
+      <c r="C76" s="14" t="s">
         <v>264</v>
       </c>
-      <c r="C76" s="14" t="s">
+      <c r="D76" t="s">
         <v>265</v>
       </c>
-      <c r="D76" t="s">
-        <v>266</v>
-      </c>
       <c r="E76" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G76" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H76" s="14"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A77" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B77" s="14" t="s">
+        <v>266</v>
+      </c>
+      <c r="C77" s="14" t="s">
         <v>267</v>
       </c>
-      <c r="C77" s="14" t="s">
+      <c r="D77" t="s">
         <v>268</v>
       </c>
-      <c r="D77" t="s">
-        <v>269</v>
-      </c>
       <c r="E77" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="F77" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G77" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H77" s="14"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B78" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="C78" s="14" t="s">
         <v>270</v>
       </c>
-      <c r="C78" s="14" t="s">
+      <c r="D78" t="s">
         <v>271</v>
       </c>
-      <c r="D78" t="s">
-        <v>272</v>
-      </c>
       <c r="E78" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="F78" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G78" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H78" s="14"/>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A79" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B79" s="14" t="s">
+        <v>272</v>
+      </c>
+      <c r="C79" s="14" t="s">
         <v>273</v>
       </c>
-      <c r="C79" s="14" t="s">
+      <c r="D79" t="s">
         <v>274</v>
       </c>
-      <c r="D79" t="s">
-        <v>275</v>
-      </c>
       <c r="E79" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F79" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G79" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H79" s="14"/>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A80" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B80" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="C80" s="14" t="s">
         <v>276</v>
       </c>
-      <c r="C80" s="14" t="s">
+      <c r="D80" t="s">
         <v>277</v>
       </c>
-      <c r="D80" t="s">
-        <v>278</v>
-      </c>
       <c r="E80" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="F80" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G80" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H80" s="14"/>
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B81" s="14" t="s">
+        <v>278</v>
+      </c>
+      <c r="C81" s="14" t="s">
         <v>279</v>
       </c>
-      <c r="C81" s="14" t="s">
+      <c r="D81" t="s">
         <v>280</v>
       </c>
-      <c r="D81" t="s">
-        <v>281</v>
-      </c>
       <c r="E81" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F81" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G81" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H81" s="14"/>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B82" s="14" t="s">
+        <v>281</v>
+      </c>
+      <c r="C82" s="14" t="s">
         <v>282</v>
       </c>
-      <c r="C82" s="14" t="s">
+      <c r="D82" t="s">
         <v>283</v>
       </c>
-      <c r="D82" t="s">
-        <v>284</v>
-      </c>
       <c r="E82" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F82" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G82" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H82" s="14"/>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B83" s="14" t="s">
+        <v>284</v>
+      </c>
+      <c r="C83" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="C83" s="14" t="s">
+      <c r="D83" t="s">
         <v>286</v>
       </c>
-      <c r="D83" t="s">
-        <v>287</v>
-      </c>
       <c r="E83" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F83" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G83" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H83" s="14"/>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A84" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B84" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="C84" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="C84" s="14" t="s">
+      <c r="D84" t="s">
         <v>289</v>
       </c>
-      <c r="D84" t="s">
-        <v>290</v>
-      </c>
       <c r="E84" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="F84" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G84" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H84" s="14"/>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A85" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B85" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="C85" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="C85" s="14" t="s">
+      <c r="D85" t="s">
         <v>292</v>
       </c>
-      <c r="D85" t="s">
-        <v>293</v>
-      </c>
       <c r="E85" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F85" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G85" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H85" s="14"/>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B86" s="14" t="s">
+        <v>293</v>
+      </c>
+      <c r="C86" s="14" t="s">
         <v>294</v>
       </c>
-      <c r="C86" s="14" t="s">
+      <c r="D86" t="s">
         <v>295</v>
       </c>
-      <c r="D86" t="s">
-        <v>296</v>
-      </c>
       <c r="E86" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F86" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G86" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H86" s="14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A87" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B87" s="14" t="s">
+        <v>296</v>
+      </c>
+      <c r="C87" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="C87" s="14" t="s">
+      <c r="D87" t="s">
         <v>298</v>
       </c>
-      <c r="D87" t="s">
-        <v>299</v>
-      </c>
       <c r="E87" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F87" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G87" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H87" s="14"/>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B88" s="14" t="s">
+        <v>299</v>
+      </c>
+      <c r="C88" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="C88" s="14" t="s">
+      <c r="D88" t="s">
         <v>301</v>
       </c>
-      <c r="D88" t="s">
-        <v>302</v>
-      </c>
       <c r="E88" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F88" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G88" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H88" s="14"/>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B89" s="14" t="s">
+        <v>302</v>
+      </c>
+      <c r="C89" s="14" t="s">
         <v>303</v>
       </c>
-      <c r="C89" s="14" t="s">
+      <c r="D89" t="s">
         <v>304</v>
       </c>
-      <c r="D89" t="s">
-        <v>305</v>
-      </c>
       <c r="E89" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="F89" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G89" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H89" s="14"/>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B90" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="C90" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="C90" s="14" t="s">
+      <c r="D90" t="s">
         <v>307</v>
       </c>
-      <c r="D90" t="s">
-        <v>308</v>
-      </c>
       <c r="E90" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F90" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G90" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H90" s="14"/>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B91" s="14" t="s">
+        <v>308</v>
+      </c>
+      <c r="C91" s="14" t="s">
         <v>309</v>
       </c>
-      <c r="C91" s="14" t="s">
+      <c r="D91" t="s">
         <v>310</v>
       </c>
-      <c r="D91" t="s">
-        <v>311</v>
-      </c>
       <c r="E91" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F91" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G91" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H91" s="14"/>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B92" s="14" t="s">
+        <v>311</v>
+      </c>
+      <c r="C92" s="14" t="s">
         <v>312</v>
       </c>
-      <c r="C92" s="14" t="s">
+      <c r="D92" t="s">
         <v>313</v>
       </c>
-      <c r="D92" t="s">
-        <v>314</v>
-      </c>
       <c r="E92" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F92" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G92" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H92" s="14"/>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B93" s="14" t="s">
+        <v>314</v>
+      </c>
+      <c r="C93" s="14" t="s">
         <v>315</v>
       </c>
-      <c r="C93" s="14" t="s">
+      <c r="D93" t="s">
         <v>316</v>
       </c>
-      <c r="D93" t="s">
-        <v>317</v>
-      </c>
       <c r="E93" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F93" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G93" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H93" s="14"/>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B94" s="14" t="s">
+        <v>317</v>
+      </c>
+      <c r="C94" s="14" t="s">
         <v>318</v>
       </c>
-      <c r="C94" s="14" t="s">
+      <c r="D94" t="s">
         <v>319</v>
       </c>
-      <c r="D94" t="s">
-        <v>320</v>
-      </c>
       <c r="E94" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F94" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G94" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H94" s="14"/>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A95" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B95" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="C95" s="14" t="s">
         <v>321</v>
       </c>
-      <c r="C95" s="14" t="s">
+      <c r="D95" t="s">
         <v>322</v>
       </c>
-      <c r="D95" t="s">
-        <v>323</v>
-      </c>
       <c r="E95" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F95" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G95" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H95" s="14"/>
     </row>
     <row r="96" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A96" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B96" s="14" t="s">
+        <v>323</v>
+      </c>
+      <c r="C96" s="14" t="s">
         <v>324</v>
       </c>
-      <c r="C96" s="14" t="s">
+      <c r="D96" t="s">
         <v>325</v>
       </c>
-      <c r="D96" t="s">
-        <v>326</v>
-      </c>
       <c r="E96" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F96" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G96" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H96" s="14"/>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B97" s="14" t="s">
+        <v>326</v>
+      </c>
+      <c r="C97" s="14" t="s">
         <v>327</v>
       </c>
-      <c r="C97" s="14" t="s">
+      <c r="D97" t="s">
         <v>328</v>
       </c>
-      <c r="D97" t="s">
-        <v>329</v>
-      </c>
       <c r="E97" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="F97" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G97" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H97" s="14"/>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B98" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="C98" s="14" t="s">
         <v>330</v>
       </c>
-      <c r="C98" s="14" t="s">
+      <c r="D98" t="s">
         <v>331</v>
       </c>
-      <c r="D98" t="s">
-        <v>332</v>
-      </c>
       <c r="E98" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="F98" s="15" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G98" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H98" s="14"/>
     </row>
@@ -6990,30 +7008,30 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C2">
         <v>-33.599203000000003</v>
@@ -7030,10 +7048,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B3" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C3">
         <v>-33.599203000000003</v>
@@ -7050,10 +7068,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C4">
         <v>-33.599203000000003</v>
@@ -7070,10 +7088,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C5">
         <v>-33.599203000000003</v>
@@ -7090,10 +7108,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B6" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C6">
         <v>-33.599203000000003</v>
@@ -7110,10 +7128,10 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C7">
         <v>-33.599203000000003</v>
@@ -7130,10 +7148,10 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C8">
         <v>-33.599203000000003</v>
@@ -7150,10 +7168,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C9">
         <v>-33.599203000000003</v>
@@ -7170,10 +7188,10 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B10" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C10">
         <v>-33.599203000000003</v>
@@ -7190,10 +7208,10 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C11">
         <v>-33.599203000000003</v>
@@ -7663,7 +7681,7 @@
   <sheetPr>
     <tabColor rgb="FFFF3838"/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="14.33203125" customWidth="1"/>
@@ -7673,65 +7691,68 @@
     <col min="6" max="6" width="30.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="48" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A1" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="12" t="s">
-        <v>39</v>
-      </c>
       <c r="C1" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="D1" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="E1" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>352</v>
+      </c>
+      <c r="H1" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>354</v>
+      </c>
+      <c r="J1" s="29" t="s">
+        <v>346</v>
+      </c>
+      <c r="K1" s="29" t="s">
+        <v>355</v>
+      </c>
+      <c r="L1" s="29" t="s">
+        <v>356</v>
+      </c>
+      <c r="M1" s="29" t="s">
+        <v>357</v>
+      </c>
+      <c r="N1" s="29" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A2" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C2" s="14" t="s">
         <v>335</v>
       </c>
-      <c r="E1" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="18" t="s">
-        <v>353</v>
-      </c>
-      <c r="H1" s="18" t="s">
-        <v>354</v>
-      </c>
-      <c r="I1" s="18" t="s">
-        <v>355</v>
-      </c>
-      <c r="J1" s="29" t="s">
-        <v>347</v>
-      </c>
-      <c r="K1" s="29" t="s">
-        <v>357</v>
-      </c>
-      <c r="L1" s="29" t="s">
+      <c r="D2" s="14" t="s">
+        <v>336</v>
+      </c>
+      <c r="E2" s="19" t="s">
+        <v>337</v>
+      </c>
+      <c r="F2" s="20" t="s">
         <v>358</v>
-      </c>
-      <c r="M1" s="29" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B2" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" s="14" t="s">
-        <v>336</v>
-      </c>
-      <c r="D2" s="14" t="s">
-        <v>337</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>338</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>360</v>
       </c>
       <c r="G2" s="19">
         <v>640</v>
@@ -7753,6 +7774,9 @@
       </c>
       <c r="M2" s="14">
         <v>2.2999999999999998</v>
+      </c>
+      <c r="N2" s="14" t="s">
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>